<commit_message>
Upload GitHub Summary - 2025-06-09 14:32:49
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -481,7 +481,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2877</v>
+        <v>626</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -504,7 +504,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="C3">
         <v>7</v>
@@ -527,7 +527,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -550,7 +550,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>74</v>
+        <v>31</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -573,7 +573,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>239</v>
+        <v>64</v>
       </c>
       <c r="C6">
         <v>8</v>
@@ -596,7 +596,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>159</v>
+        <v>57</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -624,7 +624,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>130</v>
+        <v>83</v>
       </c>
       <c r="C9">
         <v>20</v>
@@ -652,7 +652,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>626</v>
+        <v>2881</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -736,7 +736,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="C3">
         <v>12</v>
@@ -759,7 +759,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -782,7 +782,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>31</v>
+        <v>74</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -805,7 +805,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>64</v>
+        <v>239</v>
       </c>
       <c r="C6">
         <v>40</v>
@@ -828,7 +828,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>57</v>
+        <v>159</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -856,7 +856,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>83</v>
+        <v>130</v>
       </c>
       <c r="C9">
         <v>54</v>
@@ -884,7 +884,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="C11">
         <v>0</v>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-10 19:20:06
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2881</v>
+        <v>2882</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-12 01:31:20
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -481,7 +481,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -496,7 +496,7 @@
         <v>87</v>
       </c>
       <c r="G2">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2882</v>
+        <v>2883</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-13 01:35:37
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -481,7 +481,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -496,7 +496,7 @@
         <v>87</v>
       </c>
       <c r="G2">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2883</v>
+        <v>2886</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-14 01:31:18
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2886</v>
+        <v>2888</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-17 01:31:29
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2888</v>
+        <v>2890</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-18 01:31:26
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2890</v>
+        <v>2891</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-19 01:31:29
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2891</v>
+        <v>2892</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-20 01:31:31
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2892</v>
+        <v>2893</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-21 01:31:03
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2893</v>
+        <v>2897</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>224</v>
+        <v>228</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -884,7 +884,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -899,7 +899,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-24 01:31:31
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -573,7 +573,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C6">
         <v>8</v>
@@ -588,7 +588,7 @@
         <v>11</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2897</v>
+        <v>2898</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -805,7 +805,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C6">
         <v>40</v>
@@ -820,7 +820,7 @@
         <v>14</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -828,7 +828,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -843,7 +843,7 @@
         <v>38</v>
       </c>
       <c r="G7">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -884,7 +884,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -899,7 +899,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-25 01:31:27
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2898</v>
+        <v>2899</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-26 01:31:21
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2899</v>
+        <v>2900</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-27 01:31:26
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2900</v>
+        <v>2903</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-06-28 01:31:02
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2903</v>
+        <v>2908</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>234</v>
+        <v>239</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-02 01:31:30
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2908</v>
+        <v>2909</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-04 01:31:25
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -481,7 +481,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -496,7 +496,7 @@
         <v>87</v>
       </c>
       <c r="G2">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2909</v>
+        <v>2913</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>240</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-08 01:31:37
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2913</v>
+        <v>2914</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-09 01:31:36
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2914</v>
+        <v>2915</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-10 01:31:35
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2915</v>
+        <v>2916</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-11 01:31:48
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2916</v>
+        <v>2917</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-12 01:31:53
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2917</v>
+        <v>2918</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-15 01:32:09
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2918</v>
+        <v>2920</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-17 01:31:52
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -652,7 +652,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -667,7 +667,7 @@
         <v>1</v>
       </c>
       <c r="G11">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -884,7 +884,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -899,7 +899,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-18 01:32:32
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2920</v>
+        <v>2921</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-19 01:31:34
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -884,7 +884,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -899,7 +899,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-24 14:00:15
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -481,7 +481,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -496,7 +496,7 @@
         <v>87</v>
       </c>
       <c r="G2">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2921</v>
+        <v>2925</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-25 02:54:52
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2925</v>
+        <v>2926</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-26 02:49:31
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2926</v>
+        <v>2927</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-29 03:06:43
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -504,19 +504,19 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="C3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2927</v>
+        <v>2928</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -736,19 +736,19 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>77</v>
+        <v>26</v>
       </c>
       <c r="C3">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D3">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G3">
         <v>1</v>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-30 02:59:05
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -481,7 +481,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -496,7 +496,7 @@
         <v>87</v>
       </c>
       <c r="G2">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -504,19 +504,19 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2928</v>
+        <v>2929</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -736,19 +736,19 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>26</v>
+        <v>77</v>
       </c>
       <c r="C3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G3">
         <v>1</v>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-07-31 02:58:31
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2929</v>
+        <v>2930</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-08-01 03:09:40
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2930</v>
+        <v>2931</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-08-02 02:50:39
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2931</v>
+        <v>2932</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-08-05 03:01:52
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2932</v>
+        <v>2935</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-08-13 02:46:13
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -481,7 +481,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -496,7 +496,7 @@
         <v>87</v>
       </c>
       <c r="G2">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2935</v>
+        <v>2937</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-08-14 02:47:18
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2937</v>
+        <v>2938</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-08-15 02:48:30
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -481,7 +481,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -496,7 +496,7 @@
         <v>87</v>
       </c>
       <c r="G2">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2938</v>
+        <v>2941</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-08-20 02:27:55
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2941</v>
+        <v>2943</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-08-21 02:27:07
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2943</v>
+        <v>2944</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -828,7 +828,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -843,7 +843,7 @@
         <v>38</v>
       </c>
       <c r="G7">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-08-29 02:23:26
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2944</v>
+        <v>2945</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-08-30 02:17:34
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2945</v>
+        <v>2948</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-09-02 02:25:39
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2941</v>
+        <v>2948</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>272</v>
+        <v>279</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -828,7 +828,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -843,7 +843,7 @@
         <v>38</v>
       </c>
       <c r="G7">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-09-03 02:16:56
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2948</v>
+        <v>2955</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>279</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-09-10 02:16:53
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2955</v>
+        <v>2957</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-09-11 02:21:05
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -713,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2957</v>
+        <v>2958</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -728,7 +728,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-09-11 22:58:05
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -10,13 +10,14 @@
     <sheet name="Unique users" sheetId="1" r:id="rId1"/>
     <sheet name="User issues" sheetId="2" r:id="rId2"/>
     <sheet name="vendor-mapping" sheetId="3" r:id="rId3"/>
+    <sheet name="metainfo" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
   <si>
     <t>Ecosystem</t>
   </si>
@@ -88,6 +89,18 @@
   </si>
   <si>
     <t>mostly-ai</t>
+  </si>
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>September 11, 2025</t>
   </si>
 </sst>
 </file>
@@ -985,4 +998,34 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="7.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-09-12 02:15:59
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 11, 2025</t>
+    <t>September 12, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2958</v>
+        <v>2959</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -897,7 +897,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -912,7 +912,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-09-16 02:17:50
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 15, 2025</t>
+    <t>September 16, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2959</v>
+        <v>2961</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -897,7 +897,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -912,7 +912,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-09-26 02:20:37
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 25, 2025</t>
+    <t>September 26, 2025</t>
   </si>
 </sst>
 </file>
@@ -897,7 +897,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -912,7 +912,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-09-30 02:18:16
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 29, 2025</t>
+    <t>September 30, 2025</t>
   </si>
 </sst>
 </file>
@@ -609,7 +609,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -624,7 +624,7 @@
         <v>25</v>
       </c>
       <c r="G7">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -665,7 +665,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -680,7 +680,7 @@
         <v>1</v>
       </c>
       <c r="G11">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2961</v>
+        <v>2963</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -841,7 +841,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -856,7 +856,7 @@
         <v>38</v>
       </c>
       <c r="G7">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -897,7 +897,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -912,7 +912,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-01 02:29:42
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 30, 2025</t>
+    <t>October 1, 2025</t>
   </si>
 </sst>
 </file>
@@ -665,7 +665,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -680,7 +680,7 @@
         <v>1</v>
       </c>
       <c r="G11">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -897,7 +897,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -912,7 +912,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1006,7 +1006,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-02 02:17:59
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 1, 2025</t>
+    <t>October 2, 2025</t>
   </si>
 </sst>
 </file>
@@ -609,7 +609,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -624,7 +624,7 @@
         <v>25</v>
       </c>
       <c r="G7">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2963</v>
+        <v>2969</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>294</v>
+        <v>300</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -841,7 +841,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -856,7 +856,7 @@
         <v>38</v>
       </c>
       <c r="G7">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-03 02:17:39
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 2, 2025</t>
+    <t>October 3, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2969</v>
+        <v>2971</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-04 02:12:35
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 3, 2025</t>
+    <t>October 4, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2971</v>
+        <v>2972</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -897,7 +897,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -912,7 +912,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-05 02:27:32
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 4, 2025</t>
+    <t>October 5, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2972</v>
+        <v>2973</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-06 03:36:46
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 5, 2025</t>
+    <t>October 6, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2973</v>
+        <v>2977</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>304</v>
+        <v>308</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-07 02:18:44
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 6, 2025</t>
+    <t>October 7, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2977</v>
+        <v>2979</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-09 02:20:09
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 8, 2025</t>
+    <t>October 9, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2979</v>
+        <v>2981</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-10 02:20:39
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 9, 2025</t>
+    <t>October 10, 2025</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1006,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-11 02:15:30
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 10, 2025</t>
+    <t>October 11, 2025</t>
   </si>
 </sst>
 </file>
@@ -494,7 +494,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -509,7 +509,7 @@
         <v>87</v>
       </c>
       <c r="G2">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2981</v>
+        <v>2983</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-14 02:20:49
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 13, 2025</t>
+    <t>October 14, 2025</t>
   </si>
 </sst>
 </file>
@@ -494,7 +494,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -509,7 +509,7 @@
         <v>87</v>
       </c>
       <c r="G2">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2983</v>
+        <v>2985</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-15 02:23:53
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 14, 2025</t>
+    <t>October 15, 2025</t>
   </si>
 </sst>
 </file>
@@ -609,7 +609,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -624,7 +624,7 @@
         <v>25</v>
       </c>
       <c r="G7">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2985</v>
+        <v>2990</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>316</v>
+        <v>321</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -841,7 +841,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -856,7 +856,7 @@
         <v>38</v>
       </c>
       <c r="G7">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-16 02:22:20
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 15, 2025</t>
+    <t>October 16, 2025</t>
   </si>
 </sst>
 </file>
@@ -609,7 +609,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -624,7 +624,7 @@
         <v>25</v>
       </c>
       <c r="G7">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2990</v>
+        <v>2992</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -841,7 +841,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -856,7 +856,7 @@
         <v>38</v>
       </c>
       <c r="G7">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-17 02:21:52
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 16, 2025</t>
+    <t>October 17, 2025</t>
   </si>
 </sst>
 </file>
@@ -841,7 +841,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -856,7 +856,7 @@
         <v>38</v>
       </c>
       <c r="G7">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-18 02:16:07
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 17, 2025</t>
+    <t>October 18, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2992</v>
+        <v>2993</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-21 02:25:26
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 20, 2025</t>
+    <t>October 21, 2025</t>
   </si>
 </sst>
 </file>
@@ -637,7 +637,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C9">
         <v>20</v>
@@ -652,7 +652,7 @@
         <v>16</v>
       </c>
       <c r="G9">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2993</v>
+        <v>2995</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -869,7 +869,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C9">
         <v>54</v>
@@ -884,7 +884,7 @@
         <v>17</v>
       </c>
       <c r="G9">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-22 02:28:19
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 21, 2025</t>
+    <t>October 22, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2995</v>
+        <v>3004</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>326</v>
+        <v>335</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -897,7 +897,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -912,7 +912,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-29 02:42:38
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 27, 2025</t>
+    <t>October 29, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3004</v>
+        <v>3010</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>335</v>
+        <v>341</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-10-31 02:28:00
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 30, 2025</t>
+    <t>October 31, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3010</v>
+        <v>3012</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-01 02:29:28
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 31, 2025</t>
+    <t>November 1, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3012</v>
+        <v>3015</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>343</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-04 02:27:38
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 3, 2025</t>
+    <t>November 4, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3015</v>
+        <v>3018</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>346</v>
+        <v>349</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-05 02:29:23
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 4, 2025</t>
+    <t>November 5, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3018</v>
+        <v>3019</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-07 02:27:55
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 6, 2025</t>
+    <t>November 7, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3019</v>
+        <v>3023</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>350</v>
+        <v>354</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-08 02:21:18
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 7, 2025</t>
+    <t>November 8, 2025</t>
   </si>
 </sst>
 </file>
@@ -665,7 +665,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -680,7 +680,7 @@
         <v>1</v>
       </c>
       <c r="G11">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -897,7 +897,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -912,7 +912,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-10 03:09:05
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 9, 2025</t>
+    <t>November 10, 2025</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1006,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-12 02:28:43
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 11, 2025</t>
+    <t>November 12, 2025</t>
   </si>
 </sst>
 </file>
@@ -897,7 +897,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -912,7 +912,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-13 02:42:09
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 12, 2025</t>
+    <t>November 13, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3023</v>
+        <v>3024</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-14 02:29:24
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 13, 2025</t>
+    <t>November 14, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3024</v>
+        <v>3025</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-15 02:24:58
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 14, 2025</t>
+    <t>November 15, 2025</t>
   </si>
 </sst>
 </file>
@@ -494,7 +494,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -509,7 +509,7 @@
         <v>87</v>
       </c>
       <c r="G2">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3025</v>
+        <v>3027</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -841,7 +841,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -856,7 +856,7 @@
         <v>38</v>
       </c>
       <c r="G7">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-18 02:29:01
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 17, 2025</t>
+    <t>November 18, 2025</t>
   </si>
 </sst>
 </file>
@@ -494,7 +494,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -509,7 +509,7 @@
         <v>87</v>
       </c>
       <c r="G2">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3027</v>
+        <v>3029</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-19 02:28:28
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 18, 2025</t>
+    <t>November 19, 2025</t>
   </si>
 </sst>
 </file>
@@ -897,7 +897,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -912,7 +912,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-22 02:22:40
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 21, 2025</t>
+    <t>November 22, 2025</t>
   </si>
 </sst>
 </file>
@@ -772,7 +772,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -787,7 +787,7 @@
         <v>11</v>
       </c>
       <c r="G4">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-25 02:41:56
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 24, 2025</t>
+    <t>November 25, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3029</v>
+        <v>3030</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-29 02:27:14
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 28, 2025</t>
+    <t>November 29, 2025</t>
   </si>
 </sst>
 </file>
@@ -609,7 +609,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -624,7 +624,7 @@
         <v>25</v>
       </c>
       <c r="G7">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -841,7 +841,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -856,7 +856,7 @@
         <v>38</v>
       </c>
       <c r="G7">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-11-30 02:53:27
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 29, 2025</t>
+    <t>November 30, 2025</t>
   </si>
 </sst>
 </file>
@@ -772,7 +772,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -787,7 +787,7 @@
         <v>11</v>
       </c>
       <c r="G4">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-12-01 03:04:37
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>November 30, 2025</t>
+    <t>December 1, 2025</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1006,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-12-02 02:44:44
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>December 1, 2025</t>
+    <t>December 2, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3030</v>
+        <v>3031</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-12-03 02:43:54
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>December 2, 2025</t>
+    <t>December 3, 2025</t>
   </si>
 </sst>
 </file>
@@ -494,7 +494,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -509,7 +509,7 @@
         <v>87</v>
       </c>
       <c r="G2">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3031</v>
+        <v>3032</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-12-05 02:45:46
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>December 4, 2025</t>
+    <t>December 5, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3032</v>
+        <v>3033</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-12-09 02:44:55
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>December 8, 2025</t>
+    <t>December 9, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3033</v>
+        <v>3034</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-12-10 02:48:44
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>December 9, 2025</t>
+    <t>December 10, 2025</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1006,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-12-11 02:50:20
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>December 10, 2025</t>
+    <t>December 11, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3034</v>
+        <v>3035</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-12-18 02:46:35
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>December 17, 2025</t>
+    <t>December 18, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3035</v>
+        <v>3037</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-12-20 02:29:56
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>December 19, 2025</t>
+    <t>December 20, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3037</v>
+        <v>3039</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-12-23 02:51:45
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>December 22, 2025</t>
+    <t>December 23, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3039</v>
+        <v>3042</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-12-24 02:49:06
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>December 23, 2025</t>
+    <t>December 24, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3042</v>
+        <v>3044</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2025-12-31 02:52:07
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>December 30, 2025</t>
+    <t>December 31, 2025</t>
   </si>
 </sst>
 </file>
@@ -726,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3044</v>
+        <v>3045</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -741,7 +741,7 @@
         <v>547</v>
       </c>
       <c r="G2">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="3" spans="1:7">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-01-01 03:04:21
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>December 31, 2025</t>
+    <t>January 1, 2026</t>
   </si>
 </sst>
 </file>
@@ -458,15 +458,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="23.7109375" customWidth="1"/>
-    <col min="3" max="7" width="6.7109375" customWidth="1"/>
+    <col min="3" max="8" width="6.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -488,8 +488,11 @@
       <c r="G1" s="1">
         <v>2025</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -511,8 +514,11 @@
       <c r="G2">
         <v>46</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="H2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -534,8 +540,11 @@
       <c r="G3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="H3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -557,8 +566,11 @@
       <c r="G4">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="H4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -580,8 +592,11 @@
       <c r="G5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="H5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -603,8 +618,11 @@
       <c r="G6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="H6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -626,13 +644,16 @@
       <c r="G7">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="H7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -654,13 +675,16 @@
       <c r="G9">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="H9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -681,6 +705,9 @@
       </c>
       <c r="G11">
         <v>12</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -690,15 +717,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="23.7109375" customWidth="1"/>
-    <col min="3" max="7" width="6.7109375" customWidth="1"/>
+    <col min="3" max="8" width="6.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -720,8 +747,11 @@
       <c r="G1" s="1">
         <v>2025</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -743,8 +773,11 @@
       <c r="G2">
         <v>376</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="H2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -766,8 +799,11 @@
       <c r="G3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="H3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -789,8 +825,11 @@
       <c r="G4">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="H4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -812,8 +851,11 @@
       <c r="G5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="H5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -835,8 +877,11 @@
       <c r="G6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="H6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -858,13 +903,16 @@
       <c r="G7">
         <v>23</v>
       </c>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="H7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -886,13 +934,16 @@
       <c r="G9">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="H9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -913,6 +964,9 @@
       </c>
       <c r="G11">
         <v>48</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1006,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-01-22 17:27:08
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>January 2, 2026</t>
+    <t>January 22, 2026</t>
   </si>
 </sst>
 </file>
@@ -575,7 +575,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>2</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -627,7 +627,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -645,7 +645,7 @@
         <v>13</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3045</v>
+        <v>3075</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -834,7 +834,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -852,7 +852,7 @@
         <v>2</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -886,7 +886,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -904,7 +904,7 @@
         <v>23</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-01-23 03:00:50
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>January 22, 2026</t>
+    <t>January 23, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3075</v>
+        <v>3077</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-01-24 02:55:15
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>January 23, 2026</t>
+    <t>January 24, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3077</v>
+        <v>3083</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-01-26 03:16:20
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>January 25, 2026</t>
+    <t>January 26, 2026</t>
   </si>
 </sst>
 </file>
@@ -601,7 +601,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C6">
         <v>8</v>
@@ -619,7 +619,7 @@
         <v>1</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -860,7 +860,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C6">
         <v>40</v>
@@ -878,7 +878,7 @@
         <v>1</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-01-27 03:06:15
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>January 26, 2026</t>
+    <t>January 27, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3083</v>
+        <v>3085</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-01-28 03:03:35
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>January 27, 2026</t>
+    <t>January 28, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3085</v>
+        <v>3088</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-01-29 03:27:18
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>January 28, 2026</t>
+    <t>January 29, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3088</v>
+        <v>3093</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-01-31 03:22:56
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>January 30, 2026</t>
+    <t>January 31, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3093</v>
+        <v>3096</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-02-01 03:49:04
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>January 31, 2026</t>
+    <t>February 1, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3096</v>
+        <v>3097</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-02-05 03:33:21
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>February 4, 2026</t>
+    <t>February 5, 2026</t>
   </si>
 </sst>
 </file>
@@ -497,7 +497,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -515,7 +515,7 @@
         <v>46</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -601,7 +601,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C6">
         <v>8</v>
@@ -619,7 +619,7 @@
         <v>1</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3097</v>
+        <v>3104</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -860,7 +860,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C6">
         <v>40</v>
@@ -878,7 +878,7 @@
         <v>1</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-02-08 03:54:31
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>February 7, 2026</t>
+    <t>February 8, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3104</v>
+        <v>3105</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-02-10 03:51:12
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>February 9, 2026</t>
+    <t>February 10, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3105</v>
+        <v>3107</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-02-14 03:28:34
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>February 13, 2026</t>
+    <t>February 14, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3107</v>
+        <v>3110</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-02-17 03:36:05
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>February 16, 2026</t>
+    <t>February 17, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3110</v>
+        <v>3111</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-02-18 03:38:34
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>February 17, 2026</t>
+    <t>February 18, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3111</v>
+        <v>3114</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-02-19 03:37:30
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>February 18, 2026</t>
+    <t>February 19, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3114</v>
+        <v>3115</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-02-24 03:36:22
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>February 23, 2026</t>
+    <t>February 24, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3115</v>
+        <v>3120</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-02-25 03:36:33
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>February 24, 2026</t>
+    <t>February 25, 2026</t>
   </si>
 </sst>
 </file>
@@ -601,7 +601,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C6">
         <v>8</v>
@@ -619,7 +619,7 @@
         <v>1</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -860,7 +860,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C6">
         <v>40</v>
@@ -878,7 +878,7 @@
         <v>1</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-02-26 03:33:41
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>February 25, 2026</t>
+    <t>February 26, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3120</v>
+        <v>3124</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-02-28 03:10:43
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>February 27, 2026</t>
+    <t>February 28, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3124</v>
+        <v>3125</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-03-01 03:41:48
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>February 28, 2026</t>
+    <t>March 1, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3125</v>
+        <v>3126</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-03-06 03:27:20
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>March 5, 2026</t>
+    <t>March 6, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3126</v>
+        <v>3127</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -917,7 +917,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C9">
         <v>54</v>
@@ -935,7 +935,7 @@
         <v>4</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-03-10 03:27:13
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>March 9, 2026</t>
+    <t>March 10, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3127</v>
+        <v>3130</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-03-11 03:26:26
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>March 10, 2026</t>
+    <t>March 11, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3130</v>
+        <v>3131</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-03-21 03:22:53
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>March 20, 2026</t>
+    <t>March 21, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3131</v>
+        <v>3132</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-03-30 15:01:09
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>March 24, 2026</t>
+    <t>March 30, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3132</v>
+        <v>3136</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-04-01 04:15:33
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>March 31, 2026</t>
+    <t>April 1, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3136</v>
+        <v>3137</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-04-02 03:48:13
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>April 1, 2026</t>
+    <t>April 2, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3137</v>
+        <v>3139</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-04-07 03:52:47
</commit_message>
<xml_diff>
--- a/assets/GitHub_Summary.xlsx
+++ b/assets/GitHub_Summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>April 6, 2026</t>
+    <t>April 7, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3139</v>
+        <v>3141</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>